<commit_message>
Vorbereitung der Zusammenführung Standard / Light
git-svn-id: svn://svn.code.sf.net/p/itelex/code-0/branch/22-04_Light@941 eda8b1fe-747e-4470-9eba-51160ea1b311
</commit_message>
<xml_diff>
--- a/AvrNetIO-Anschluesse.xlsx
+++ b/AvrNetIO-Anschluesse.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Daten\AvrProgs\i-Telex\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BD679CD-EBB4-4D59-B054-42F568BC6D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8338379-A391-4DE8-B0BC-1EB2D5EFFF93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25080" yWindow="-645" windowWidth="29040" windowHeight="15840" xr2:uid="{DAF96758-D4CB-483D-B41C-05E3EF715EF6}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="84">
   <si>
     <t>ATmegaXX4</t>
   </si>
@@ -204,12 +204,6 @@
     <t>D7</t>
   </si>
   <si>
-    <t>an ENC, auch ISP input</t>
-  </si>
-  <si>
-    <t>an ENC</t>
-  </si>
-  <si>
     <t>EXT</t>
   </si>
   <si>
@@ -226,6 +220,72 @@
   </si>
   <si>
     <t>iTelex Bus A2 C2</t>
+  </si>
+  <si>
+    <t>INT(ENC)</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>an ENC 7, auch ISP input</t>
+  </si>
+  <si>
+    <t>an ENC 6, auch ISP input</t>
+  </si>
+  <si>
+    <t>an ENC 8, auch ISP input</t>
+  </si>
+  <si>
+    <t>an ENC 9</t>
+  </si>
+  <si>
+    <t>an ENC 4</t>
+  </si>
+  <si>
+    <t>ATmega2561</t>
+  </si>
+  <si>
+    <t>Signal</t>
+  </si>
+  <si>
+    <t>PIN SV4</t>
+  </si>
+  <si>
+    <t>F4</t>
+  </si>
+  <si>
+    <t>F7</t>
+  </si>
+  <si>
+    <t>F6</t>
+  </si>
+  <si>
+    <t>F5</t>
+  </si>
+  <si>
+    <t>TCK</t>
+  </si>
+  <si>
+    <t>TDI</t>
+  </si>
+  <si>
+    <t>TDO</t>
+  </si>
+  <si>
+    <t>TMS</t>
+  </si>
+  <si>
+    <t>ISP 10pol</t>
+  </si>
+  <si>
+    <t>ISP Signal</t>
+  </si>
+  <si>
+    <t>SCK</t>
+  </si>
+  <si>
+    <t>RST</t>
   </si>
 </sst>
 </file>
@@ -261,7 +321,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -274,6 +334,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -589,10 +652,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC9F4DD3-DB12-41F2-A287-6D6B18027906}">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="23" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -609,10 +673,10 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -632,7 +696,7 @@
         <v>10</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -652,7 +716,7 @@
         <v>9</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -672,7 +736,7 @@
         <v>39</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -692,7 +756,7 @@
         <v>39</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -894,7 +958,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>41</v>
       </c>
@@ -914,7 +978,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>26</v>
       </c>
@@ -931,10 +995,10 @@
         <v>39</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -951,10 +1015,10 @@
         <v>39</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -971,10 +1035,10 @@
         <v>39</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -991,87 +1055,186 @@
         <v>39</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B22" s="1">
+        <v>3</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>46</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B23" s="1">
         <v>16</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C23" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E22" s="1">
+      <c r="D23" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E23" s="1">
         <v>1</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>47</v>
-      </c>
-      <c r="B23" s="1">
-        <v>18</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E23" s="1">
-        <v>3</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H23" s="5"/>
+      <c r="I23" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="K23" s="5">
+        <v>1</v>
+      </c>
+      <c r="L23" s="5">
+        <v>1</v>
+      </c>
+      <c r="M23" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B24" s="1">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>39</v>
       </c>
       <c r="E24" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H24" s="5"/>
+      <c r="I24" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="J24" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="K24" s="5">
+        <v>9</v>
+      </c>
+      <c r="L24" s="5">
+        <v>9</v>
+      </c>
+      <c r="M24" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B25" s="1">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>39</v>
       </c>
       <c r="E25" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>51</v>
+      </c>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="K25" s="5">
+        <v>3</v>
+      </c>
+      <c r="L25" s="5">
+        <v>7</v>
+      </c>
+      <c r="M25" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" s="1">
+        <v>17</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E26" s="1">
+        <v>2</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="K26" s="5">
+        <v>5</v>
+      </c>
+      <c r="L26" s="5">
+        <v>5</v>
+      </c>
+      <c r="M26" s="5" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>